<commit_message>
Mark Super Admin / SaaS operator console tasks as In progress
17 tasks under E22 (Platform Console — SaaS Operations) whose Roles Impacted
is Platform and which the SaaS Operator Roles sheet lists Super admin as
having access to: NB-257, NB-258 through NB-273 (provisioning, tenant
lifecycle, clinic fleet/health/WABA monitoring, support tickets & access,
subscriptions/dunning, discount approvals, pricing & packaging, territory
console, multi-region residency, platform audit, usage metering).

Excluded NB-274 (Multi-branch & multi-clinic groups) despite sitting in the
same epic: its Roles Impacted is Owner, not a platform role, and its
description is clinic-owner branch management, not SaaS operator console
work.

None of this is implemented yet — status reflects that work is starting,
not that anything is built.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -25199,7 +25199,7 @@
       </c>
       <c r="R258" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S258" s="62" t="n"/>
@@ -25286,7 +25286,7 @@
       </c>
       <c r="R259" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S259" s="68" t="n"/>
@@ -25373,7 +25373,7 @@
       </c>
       <c r="R260" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S260" s="62" t="n"/>
@@ -25460,7 +25460,7 @@
       </c>
       <c r="R261" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S261" s="68" t="n"/>
@@ -25547,7 +25547,7 @@
       </c>
       <c r="R262" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S262" s="62" t="n"/>
@@ -25634,7 +25634,7 @@
       </c>
       <c r="R263" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S263" s="68" t="n"/>
@@ -25721,7 +25721,7 @@
       </c>
       <c r="R264" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S264" s="62" t="n"/>
@@ -25808,7 +25808,7 @@
       </c>
       <c r="R265" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S265" s="68" t="n"/>
@@ -25895,7 +25895,7 @@
       </c>
       <c r="R266" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S266" s="62" t="n"/>
@@ -25982,7 +25982,7 @@
       </c>
       <c r="R267" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S267" s="68" t="n"/>
@@ -26069,7 +26069,7 @@
       </c>
       <c r="R268" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S268" s="62" t="n"/>
@@ -26156,7 +26156,7 @@
       </c>
       <c r="R269" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S269" s="68" t="n"/>
@@ -26243,7 +26243,7 @@
       </c>
       <c r="R270" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S270" s="62" t="n"/>
@@ -26330,7 +26330,7 @@
       </c>
       <c r="R271" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S271" s="68" t="n"/>
@@ -26417,7 +26417,7 @@
       </c>
       <c r="R272" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S272" s="62" t="n"/>
@@ -26504,7 +26504,7 @@
       </c>
       <c r="R273" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S273" s="68" t="n"/>
@@ -26591,7 +26591,7 @@
       </c>
       <c r="R274" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S274" s="62" t="n"/>

</xml_diff>

<commit_message>
Add NB-351 for the Super Admin operator login (master schema), status Done
Mirrors the NB-350 pattern: new Backlog row plus the matching extension
of every dependent range (TOTAL row, Epics/Sprints/Tracks rollups,
status/priority/phase dropdown validations) so the row counts toward
existing summaries instead of being silently excluded.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S352"/>
+  <dimension ref="A1:S353"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="50" min="1" max="1"/>
@@ -33052,89 +33052,156 @@
       </c>
       <c r="S350" s="62" t="n"/>
     </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
+    <row r="351" s="51">
+      <c r="A351" s="50" t="inlineStr">
         <is>
           <t>NB-350</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
+      <c r="B351" s="50" t="inlineStr">
         <is>
           <t>E05 Identity, Auth &amp; Session</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr">
+      <c r="C351" s="50" t="inlineStr">
         <is>
           <t>Auth</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr">
+      <c r="D351" s="50" t="inlineStr">
         <is>
           <t>Owner account — Brand/Clinic hierarchy &amp; workspace login</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr">
+      <c r="E351" s="50" t="inlineStr">
         <is>
           <t>Owner is a new top-level account (not a row in any clinic's staff table) that owns Brand(s), each containing Clinic(s). PIN login issues a short-lived pendingToken scoped only to listing/selecting a workspace; selecting a clinic mints a normal staff-shaped access/refresh token pair via a lazily-created shadow staff row (staff.owner_id), reusing every existing clinic endpoint's RBAC checks unchanged. Clinic (tenants) remains the RLS boundary; brand-wide RLS support (app.accessible_tenant_ids) shipped at the DB layer but has no consuming dashboard endpoint yet.</t>
         </is>
       </c>
-      <c r="G351" t="inlineStr">
+      <c r="G351" s="50" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="H351" t="inlineStr">
+      <c r="H351" s="50" t="inlineStr">
         <is>
           <t>Shared</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr">
+      <c r="I351" s="50" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="J351" t="inlineStr">
+      <c r="J351" s="50" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="K351" t="inlineStr">
+      <c r="K351" s="50" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="P351" t="inlineStr">
+      <c r="P351" s="50" t="inlineStr">
         <is>
           <t>NB-040, NB-043, NB-049</t>
         </is>
       </c>
-      <c r="Q351" t="inlineStr">
+      <c r="Q351" s="50" t="inlineStr">
         <is>
           <t>Selecting a clinic the owner doesn't own returns 404, not 403; workspace listing never includes another owner's brands or clinics; the minted clinic token works unchanged against every existing staff-facing endpoint; selecting the same clinic twice reuses one shadow staff row, not a duplicate</t>
         </is>
       </c>
-      <c r="R351" t="inlineStr">
+      <c r="R351" s="50" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="352" ht="15" customHeight="1" s="51">
-      <c r="A352" s="54" t="inlineStr">
+    <row r="352" s="51">
+      <c r="A352" s="50" t="inlineStr">
+        <is>
+          <t>NB-351</t>
+        </is>
+      </c>
+      <c r="B352" s="50" t="inlineStr">
+        <is>
+          <t>E05 Identity, Auth &amp; Session</t>
+        </is>
+      </c>
+      <c r="C352" s="50" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D352" s="50" t="inlineStr">
+        <is>
+          <t>Super Admin — dedicated operator login (master schema)</t>
+        </is>
+      </c>
+      <c r="E352" s="50" t="inlineStr">
+        <is>
+          <t>Platform operators (super_admin, implementation, support_engineer, billing, sre, commercial, compliance_dpo) are a separate identity domain from clinic staff/owners, not a reserved tenant reusing staff login. master.operators/sessions/login_attempts live in a dedicated master Postgres schema, outside the tenant-scoped public schema and its RLS. PlatformAuthService mirrors the staff/owner login path's proven lockout (no self-renewal on repeated still-locked hits) and session-ownership (revoke only ever targets the caller's own session) fixes from day one, plus refresh-token rotation with family-based reuse detection and TOTP MFA. Matching /platform/login frontend page, same design tokens as /login, no clinic-code field since operators aren't tenant-scoped.</t>
+        </is>
+      </c>
+      <c r="G352" s="50" t="inlineStr">
+        <is>
+          <t>Super Admin</t>
+        </is>
+      </c>
+      <c r="H352" s="50" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="I352" s="50" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="J352" s="50" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="K352" s="50" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="P352" s="50" t="inlineStr">
+        <is>
+          <t>NB-002, NB-040</t>
+        </is>
+      </c>
+      <c r="Q352" s="50" t="inlineStr">
+        <is>
+          <t>POST /v1/platform/auth/login + /mfa/verify + /refresh + /logout + /sessions all work against master.operators, never public.staff; a still-locked login hit does not extend the lockout window; DELETE /v1/platform/auth/sessions/{id} 404s for a session owned by another operator; a reused refresh token revokes its whole family, including the token just rotated to; /platform/login renders and authenticates against a live backend</t>
+        </is>
+      </c>
+      <c r="R352" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="54" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D352" s="54">
-        <f>COUNTA(A2:A351)&amp;" tasks"</f>
-        <v/>
-      </c>
-      <c r="L352" s="54">
-        <f>SUM(L2:L351)</f>
-        <v/>
-      </c>
-      <c r="O352" s="71">
-        <f>SUM(O2:O351)</f>
+      <c r="D353" s="54">
+        <f>COUNTA(A2:A352)&amp;" tasks"</f>
+        <v/>
+      </c>
+      <c r="L353" s="54">
+        <f>SUM(L2:L352)</f>
+        <v/>
+      </c>
+      <c r="O353" s="71">
+        <f>SUM(O2:O352)</f>
         <v/>
       </c>
     </row>
@@ -33162,15 +33229,15 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="R2:R351" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="R2:R352" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Not started,In progress,Blocked,In review,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="J2:J351" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="J2:J352" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Must,Should,Could"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="K2:K351" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="K2:K352" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"MVP,Phase 2,Phase 3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -39677,11 +39744,11 @@
         </is>
       </c>
       <c r="B4" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A4)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A4)</f>
         <v/>
       </c>
       <c r="C4" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A4,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A4,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D4" s="74">
@@ -39693,39 +39760,39 @@
         <v/>
       </c>
       <c r="F4" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A4,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A4,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G4" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A4,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A4,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H4" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A4,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A4,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I4" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A4,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A4,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J4" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A4,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A4,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K4" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A4,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A4,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L4" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A4)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A4)</f>
         <v/>
       </c>
       <c r="M4" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A4)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A4)</f>
         <v/>
       </c>
       <c r="N4" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A4,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A4,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O4" s="74">
@@ -39740,11 +39807,11 @@
         </is>
       </c>
       <c r="B5" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A5)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A5,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A5,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D5" s="74">
@@ -39756,39 +39823,39 @@
         <v/>
       </c>
       <c r="F5" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A5,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A5,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G5" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A5,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A5,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H5" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A5,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A5,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I5" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A5,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A5,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J5" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A5,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A5,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K5" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A5,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A5,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L5" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A5)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A5)</f>
         <v/>
       </c>
       <c r="M5" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A5)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A5)</f>
         <v/>
       </c>
       <c r="N5" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A5,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A5,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O5" s="74">
@@ -39803,11 +39870,11 @@
         </is>
       </c>
       <c r="B6" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A6)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A6,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A6,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D6" s="74">
@@ -39819,39 +39886,39 @@
         <v/>
       </c>
       <c r="F6" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A6,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A6,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G6" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A6,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A6,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H6" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A6,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A6,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I6" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A6,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A6,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J6" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A6,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A6,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K6" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A6,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A6,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L6" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A6)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A6)</f>
         <v/>
       </c>
       <c r="M6" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A6)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A6)</f>
         <v/>
       </c>
       <c r="N6" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A6,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A6,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O6" s="74">
@@ -39866,11 +39933,11 @@
         </is>
       </c>
       <c r="B7" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A7)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A7,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A7,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D7" s="74">
@@ -39882,39 +39949,39 @@
         <v/>
       </c>
       <c r="F7" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A7,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A7,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G7" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A7,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A7,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H7" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A7,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A7,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I7" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A7,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A7,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J7" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A7,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A7,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K7" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A7,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A7,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L7" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A7)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A7)</f>
         <v/>
       </c>
       <c r="M7" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A7)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A7)</f>
         <v/>
       </c>
       <c r="N7" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A7,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A7,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O7" s="74">
@@ -39929,11 +39996,11 @@
         </is>
       </c>
       <c r="B8" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A8)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A8,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A8,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D8" s="74">
@@ -39945,39 +40012,39 @@
         <v/>
       </c>
       <c r="F8" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A8,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A8,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G8" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A8,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A8,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H8" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A8,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A8,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I8" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A8,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A8,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J8" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A8,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A8,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K8" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A8,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A8,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L8" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A8)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A8)</f>
         <v/>
       </c>
       <c r="M8" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A8)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A8)</f>
         <v/>
       </c>
       <c r="N8" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A8,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A8,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O8" s="74">
@@ -39992,11 +40059,11 @@
         </is>
       </c>
       <c r="B9" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A9)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A9,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A9,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D9" s="74">
@@ -40008,39 +40075,39 @@
         <v/>
       </c>
       <c r="F9" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A9,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A9,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G9" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A9,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A9,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H9" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A9,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A9,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I9" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A9,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A9,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J9" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A9,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A9,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K9" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A9,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A9,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L9" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A9)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A9)</f>
         <v/>
       </c>
       <c r="M9" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A9)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A9)</f>
         <v/>
       </c>
       <c r="N9" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A9,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A9,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O9" s="74">
@@ -40055,11 +40122,11 @@
         </is>
       </c>
       <c r="B10" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A10)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A10,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A10,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D10" s="74">
@@ -40071,39 +40138,39 @@
         <v/>
       </c>
       <c r="F10" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A10,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A10,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G10" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A10,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A10,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H10" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A10,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A10,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I10" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A10,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A10,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J10" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A10,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A10,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K10" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A10,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A10,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L10" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A10)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A10)</f>
         <v/>
       </c>
       <c r="M10" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A10)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A10)</f>
         <v/>
       </c>
       <c r="N10" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A10,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A10,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O10" s="74">
@@ -40118,11 +40185,11 @@
         </is>
       </c>
       <c r="B11" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A11)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A11,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A11,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D11" s="74">
@@ -40134,39 +40201,39 @@
         <v/>
       </c>
       <c r="F11" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A11,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A11,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G11" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A11,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A11,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H11" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A11,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A11,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I11" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A11,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A11,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J11" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A11,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A11,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K11" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A11,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A11,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L11" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A11)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A11)</f>
         <v/>
       </c>
       <c r="M11" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A11)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A11)</f>
         <v/>
       </c>
       <c r="N11" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A11,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A11,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O11" s="74">
@@ -40181,11 +40248,11 @@
         </is>
       </c>
       <c r="B12" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A12)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A12)</f>
         <v/>
       </c>
       <c r="C12" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A12,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A12,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D12" s="74">
@@ -40197,39 +40264,39 @@
         <v/>
       </c>
       <c r="F12" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A12,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A12,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G12" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A12,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A12,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H12" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A12,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A12,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I12" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A12,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A12,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J12" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A12,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A12,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K12" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A12,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A12,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L12" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A12)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A12)</f>
         <v/>
       </c>
       <c r="M12" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A12)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A12)</f>
         <v/>
       </c>
       <c r="N12" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A12,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A12,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O12" s="74">
@@ -40244,11 +40311,11 @@
         </is>
       </c>
       <c r="B13" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A13)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A13)</f>
         <v/>
       </c>
       <c r="C13" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A13,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A13,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D13" s="74">
@@ -40260,39 +40327,39 @@
         <v/>
       </c>
       <c r="F13" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A13,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A13,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G13" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A13,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A13,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H13" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A13,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A13,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I13" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A13,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A13,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J13" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A13,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A13,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K13" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A13,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A13,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L13" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A13)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A13)</f>
         <v/>
       </c>
       <c r="M13" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A13)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A13)</f>
         <v/>
       </c>
       <c r="N13" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A13,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A13,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O13" s="74">
@@ -40307,11 +40374,11 @@
         </is>
       </c>
       <c r="B14" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A14)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A14)</f>
         <v/>
       </c>
       <c r="C14" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A14,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A14,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D14" s="74">
@@ -40323,39 +40390,39 @@
         <v/>
       </c>
       <c r="F14" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A14,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A14,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G14" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A14,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A14,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H14" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A14,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A14,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I14" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A14,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A14,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J14" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A14,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A14,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K14" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A14,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A14,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L14" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A14)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A14)</f>
         <v/>
       </c>
       <c r="M14" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A14)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A14)</f>
         <v/>
       </c>
       <c r="N14" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A14,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A14,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O14" s="74">
@@ -40370,11 +40437,11 @@
         </is>
       </c>
       <c r="B15" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A15)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A15,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A15,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D15" s="74">
@@ -40386,39 +40453,39 @@
         <v/>
       </c>
       <c r="F15" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A15,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A15,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G15" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A15,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A15,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H15" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A15,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A15,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I15" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A15,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A15,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J15" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A15,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A15,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K15" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A15,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A15,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L15" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A15)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A15)</f>
         <v/>
       </c>
       <c r="M15" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A15)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A15)</f>
         <v/>
       </c>
       <c r="N15" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A15,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A15,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O15" s="74">
@@ -40433,11 +40500,11 @@
         </is>
       </c>
       <c r="B16" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A16)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A16,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A16,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D16" s="74">
@@ -40449,39 +40516,39 @@
         <v/>
       </c>
       <c r="F16" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A16,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A16,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G16" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A16,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A16,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H16" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A16,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A16,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I16" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A16,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A16,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J16" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A16,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A16,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K16" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A16,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A16,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L16" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A16)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A16)</f>
         <v/>
       </c>
       <c r="M16" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A16)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A16)</f>
         <v/>
       </c>
       <c r="N16" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A16,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A16,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O16" s="74">
@@ -40496,11 +40563,11 @@
         </is>
       </c>
       <c r="B17" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A17)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A17,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A17,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D17" s="74">
@@ -40512,39 +40579,39 @@
         <v/>
       </c>
       <c r="F17" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A17,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A17,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G17" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A17,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A17,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H17" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A17,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A17,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I17" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A17,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A17,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J17" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A17,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A17,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K17" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A17,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A17,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L17" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A17)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A17)</f>
         <v/>
       </c>
       <c r="M17" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A17)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A17)</f>
         <v/>
       </c>
       <c r="N17" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A17,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A17,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O17" s="74">
@@ -40559,11 +40626,11 @@
         </is>
       </c>
       <c r="B18" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A18)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A18,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A18,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D18" s="74">
@@ -40575,39 +40642,39 @@
         <v/>
       </c>
       <c r="F18" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A18,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A18,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G18" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A18,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A18,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H18" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A18,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A18,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I18" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A18,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A18,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J18" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A18,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A18,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K18" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A18,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A18,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L18" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A18)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A18)</f>
         <v/>
       </c>
       <c r="M18" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A18)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A18)</f>
         <v/>
       </c>
       <c r="N18" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A18,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A18,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O18" s="74">
@@ -40622,11 +40689,11 @@
         </is>
       </c>
       <c r="B19" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A19)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A19,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A19,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D19" s="74">
@@ -40638,39 +40705,39 @@
         <v/>
       </c>
       <c r="F19" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A19,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A19,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G19" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A19,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A19,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H19" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A19,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A19,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I19" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A19,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A19,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J19" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A19,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A19,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K19" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A19,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A19,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L19" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A19)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A19)</f>
         <v/>
       </c>
       <c r="M19" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A19)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A19)</f>
         <v/>
       </c>
       <c r="N19" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A19,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A19,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O19" s="74">
@@ -40685,11 +40752,11 @@
         </is>
       </c>
       <c r="B20" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A20)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A20,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A20,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D20" s="74">
@@ -40701,39 +40768,39 @@
         <v/>
       </c>
       <c r="F20" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A20,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A20,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G20" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A20,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A20,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H20" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A20,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A20,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I20" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A20,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A20,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J20" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A20,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A20,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K20" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A20,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A20,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L20" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A20)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A20)</f>
         <v/>
       </c>
       <c r="M20" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A20)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A20)</f>
         <v/>
       </c>
       <c r="N20" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A20,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A20,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O20" s="74">
@@ -40748,11 +40815,11 @@
         </is>
       </c>
       <c r="B21" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A21)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A21,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A21,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D21" s="74">
@@ -40764,39 +40831,39 @@
         <v/>
       </c>
       <c r="F21" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A21,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A21,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G21" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A21,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A21,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H21" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A21,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A21,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I21" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A21,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A21,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J21" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A21,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A21,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K21" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A21,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A21,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L21" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A21)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A21)</f>
         <v/>
       </c>
       <c r="M21" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A21)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A21)</f>
         <v/>
       </c>
       <c r="N21" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A21,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A21,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O21" s="74">
@@ -40811,11 +40878,11 @@
         </is>
       </c>
       <c r="B22" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A22)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A22,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A22,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D22" s="74">
@@ -40827,39 +40894,39 @@
         <v/>
       </c>
       <c r="F22" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A22,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A22,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G22" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A22,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A22,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H22" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A22,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A22,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I22" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A22,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A22,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J22" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A22,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A22,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K22" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A22,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A22,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L22" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A22)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A22)</f>
         <v/>
       </c>
       <c r="M22" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A22)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A22)</f>
         <v/>
       </c>
       <c r="N22" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A22,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A22,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O22" s="74">
@@ -40874,11 +40941,11 @@
         </is>
       </c>
       <c r="B23" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A23)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A23)</f>
         <v/>
       </c>
       <c r="C23" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A23,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A23,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D23" s="74">
@@ -40890,39 +40957,39 @@
         <v/>
       </c>
       <c r="F23" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A23,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A23,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G23" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A23,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A23,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H23" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A23,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A23,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I23" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A23,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A23,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J23" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A23,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A23,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K23" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A23,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A23,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L23" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A23)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A23)</f>
         <v/>
       </c>
       <c r="M23" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A23)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A23)</f>
         <v/>
       </c>
       <c r="N23" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A23,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A23,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O23" s="74">
@@ -40937,11 +41004,11 @@
         </is>
       </c>
       <c r="B24" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A24)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A24,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A24,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D24" s="74">
@@ -40953,39 +41020,39 @@
         <v/>
       </c>
       <c r="F24" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A24,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A24,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G24" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A24,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A24,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H24" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A24,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A24,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I24" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A24,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A24,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J24" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A24,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A24,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K24" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A24,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A24,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L24" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A24)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A24)</f>
         <v/>
       </c>
       <c r="M24" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A24)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A24)</f>
         <v/>
       </c>
       <c r="N24" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A24,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A24,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O24" s="74">
@@ -41000,11 +41067,11 @@
         </is>
       </c>
       <c r="B25" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A25)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A25,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A25,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D25" s="74">
@@ -41016,39 +41083,39 @@
         <v/>
       </c>
       <c r="F25" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A25,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A25,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G25" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A25,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A25,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H25" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A25,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A25,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I25" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A25,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A25,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J25" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A25,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A25,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K25" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A25,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A25,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L25" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A25)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A25)</f>
         <v/>
       </c>
       <c r="M25" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A25)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A25)</f>
         <v/>
       </c>
       <c r="N25" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A25,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A25,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O25" s="74">
@@ -41063,11 +41130,11 @@
         </is>
       </c>
       <c r="B26" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A26)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A26,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A26,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D26" s="74">
@@ -41079,39 +41146,39 @@
         <v/>
       </c>
       <c r="F26" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A26,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A26,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G26" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A26,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A26,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H26" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A26,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A26,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I26" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A26,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A26,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J26" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A26,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A26,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K26" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A26,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A26,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L26" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A26)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A26)</f>
         <v/>
       </c>
       <c r="M26" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A26)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A26)</f>
         <v/>
       </c>
       <c r="N26" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A26,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A26,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O26" s="74">
@@ -41126,11 +41193,11 @@
         </is>
       </c>
       <c r="B27" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A27)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A27,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A27,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D27" s="74">
@@ -41142,39 +41209,39 @@
         <v/>
       </c>
       <c r="F27" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A27,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A27,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G27" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A27,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A27,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H27" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A27,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A27,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I27" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A27,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A27,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J27" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A27,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A27,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K27" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A27,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A27,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L27" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A27)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A27)</f>
         <v/>
       </c>
       <c r="M27" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A27)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A27)</f>
         <v/>
       </c>
       <c r="N27" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A27,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A27,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O27" s="74">
@@ -41189,11 +41256,11 @@
         </is>
       </c>
       <c r="B28" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A28)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A28,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A28,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D28" s="74">
@@ -41205,39 +41272,39 @@
         <v/>
       </c>
       <c r="F28" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A28,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A28,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G28" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A28,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A28,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H28" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A28,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A28,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I28" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A28,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A28,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J28" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A28,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A28,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K28" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A28,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A28,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L28" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A28)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A28)</f>
         <v/>
       </c>
       <c r="M28" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A28)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A28)</f>
         <v/>
       </c>
       <c r="N28" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A28,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A28,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O28" s="74">
@@ -41252,11 +41319,11 @@
         </is>
       </c>
       <c r="B29" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A29)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A29,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A29,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D29" s="74">
@@ -41268,39 +41335,39 @@
         <v/>
       </c>
       <c r="F29" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A29,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A29,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G29" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A29,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A29,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H29" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A29,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A29,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I29" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A29,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A29,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J29" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A29,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A29,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K29" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A29,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A29,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L29" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A29)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A29)</f>
         <v/>
       </c>
       <c r="M29" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A29)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A29)</f>
         <v/>
       </c>
       <c r="N29" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A29,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A29,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O29" s="74">
@@ -41315,11 +41382,11 @@
         </is>
       </c>
       <c r="B30" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A30)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A30,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A30,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D30" s="74">
@@ -41331,39 +41398,39 @@
         <v/>
       </c>
       <c r="F30" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A30,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A30,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G30" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A30,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A30,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H30" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A30,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A30,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I30" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A30,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A30,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J30" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A30,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A30,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K30" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A30,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A30,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L30" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A30)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A30)</f>
         <v/>
       </c>
       <c r="M30" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A30)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A30)</f>
         <v/>
       </c>
       <c r="N30" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A30,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A30,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O30" s="74">
@@ -41378,11 +41445,11 @@
         </is>
       </c>
       <c r="B31" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A31)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A31,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A31,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D31" s="74">
@@ -41394,39 +41461,39 @@
         <v/>
       </c>
       <c r="F31" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A31,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A31,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G31" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A31,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A31,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H31" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A31,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A31,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I31" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A31,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A31,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J31" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A31,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A31,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K31" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A31,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A31,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L31" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A31)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A31)</f>
         <v/>
       </c>
       <c r="M31" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A31)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A31)</f>
         <v/>
       </c>
       <c r="N31" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A31,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A31,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O31" s="74">
@@ -41441,11 +41508,11 @@
         </is>
       </c>
       <c r="B32" s="66">
-        <f>COUNTIF(Backlog!$B$2:$B$351,$A32)</f>
+        <f>COUNTIF(Backlog!$B$2:$B$352,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="66">
-        <f>SUMIF(Backlog!$B$2:$B$351,$A32,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$B$2:$B$352,$A32,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="D32" s="74">
@@ -41457,39 +41524,39 @@
         <v/>
       </c>
       <c r="F32" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A32,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A32,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="G32" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A32,Backlog!$J$2:$J$351,"Should")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A32,Backlog!$J$2:$J$352,"Should")</f>
         <v/>
       </c>
       <c r="H32" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A32,Backlog!$J$2:$J$351,"Could")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A32,Backlog!$J$2:$J$352,"Could")</f>
         <v/>
       </c>
       <c r="I32" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A32,Backlog!$K$2:$K$351,"MVP")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A32,Backlog!$K$2:$K$352,"MVP")</f>
         <v/>
       </c>
       <c r="J32" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A32,Backlog!$K$2:$K$351,"Phase 2")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A32,Backlog!$K$2:$K$352,"Phase 2")</f>
         <v/>
       </c>
       <c r="K32" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A32,Backlog!$K$2:$K$351,"Phase 3")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A32,Backlog!$K$2:$K$352,"Phase 3")</f>
         <v/>
       </c>
       <c r="L32" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A32)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A32)</f>
         <v/>
       </c>
       <c r="M32" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$B$2:$B$351,$A32)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$B$2:$B$352,$A32)</f>
         <v/>
       </c>
       <c r="N32" s="66">
-        <f>COUNTIFS(Backlog!$B$2:$B$351,$A32,Backlog!$R$2:$R$351,"Done")</f>
+        <f>COUNTIFS(Backlog!$B$2:$B$352,$A32,Backlog!$R$2:$R$352,"Done")</f>
         <v/>
       </c>
       <c r="O32" s="74">
@@ -41683,11 +41750,11 @@
         <v/>
       </c>
       <c r="E5" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A5)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A5)</f>
         <v/>
       </c>
       <c r="F5" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A5,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A5,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G5" s="66">
@@ -41703,7 +41770,7 @@
         <v/>
       </c>
       <c r="J5" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A5,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A5,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K5" s="66">
@@ -41731,11 +41798,11 @@
         <v/>
       </c>
       <c r="E6" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A6)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A6)</f>
         <v/>
       </c>
       <c r="F6" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A6,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A6,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G6" s="66">
@@ -41751,7 +41818,7 @@
         <v/>
       </c>
       <c r="J6" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A6,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A6,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K6" s="66">
@@ -41779,11 +41846,11 @@
         <v/>
       </c>
       <c r="E7" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A7)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A7)</f>
         <v/>
       </c>
       <c r="F7" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A7,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A7,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G7" s="66">
@@ -41799,7 +41866,7 @@
         <v/>
       </c>
       <c r="J7" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A7,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A7,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K7" s="66">
@@ -41827,11 +41894,11 @@
         <v/>
       </c>
       <c r="E8" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A8)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A8)</f>
         <v/>
       </c>
       <c r="F8" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A8,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A8,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G8" s="66">
@@ -41847,7 +41914,7 @@
         <v/>
       </c>
       <c r="J8" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A8,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A8,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K8" s="66">
@@ -41875,11 +41942,11 @@
         <v/>
       </c>
       <c r="E9" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A9)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A9)</f>
         <v/>
       </c>
       <c r="F9" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A9,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A9,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G9" s="66">
@@ -41895,7 +41962,7 @@
         <v/>
       </c>
       <c r="J9" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A9,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A9,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K9" s="66">
@@ -41923,11 +41990,11 @@
         <v/>
       </c>
       <c r="E10" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A10)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A10)</f>
         <v/>
       </c>
       <c r="F10" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A10,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A10,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G10" s="66">
@@ -41943,7 +42010,7 @@
         <v/>
       </c>
       <c r="J10" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A10,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A10,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K10" s="66">
@@ -41971,11 +42038,11 @@
         <v/>
       </c>
       <c r="E11" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A11)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A11)</f>
         <v/>
       </c>
       <c r="F11" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A11,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A11,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G11" s="66">
@@ -41991,7 +42058,7 @@
         <v/>
       </c>
       <c r="J11" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A11,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A11,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K11" s="66">
@@ -42019,11 +42086,11 @@
         <v/>
       </c>
       <c r="E12" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A12)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A12)</f>
         <v/>
       </c>
       <c r="F12" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A12,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A12,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G12" s="66">
@@ -42039,7 +42106,7 @@
         <v/>
       </c>
       <c r="J12" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A12,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A12,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K12" s="66">
@@ -42067,11 +42134,11 @@
         <v/>
       </c>
       <c r="E13" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A13)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A13)</f>
         <v/>
       </c>
       <c r="F13" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A13,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A13,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G13" s="66">
@@ -42087,7 +42154,7 @@
         <v/>
       </c>
       <c r="J13" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A13,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A13,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K13" s="66">
@@ -42115,11 +42182,11 @@
         <v/>
       </c>
       <c r="E14" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A14)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A14)</f>
         <v/>
       </c>
       <c r="F14" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A14,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A14,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G14" s="66">
@@ -42135,7 +42202,7 @@
         <v/>
       </c>
       <c r="J14" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A14,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A14,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K14" s="66">
@@ -42163,11 +42230,11 @@
         <v/>
       </c>
       <c r="E15" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A15)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A15)</f>
         <v/>
       </c>
       <c r="F15" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A15,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A15,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G15" s="66">
@@ -42183,7 +42250,7 @@
         <v/>
       </c>
       <c r="J15" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A15,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A15,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K15" s="66">
@@ -42211,11 +42278,11 @@
         <v/>
       </c>
       <c r="E16" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A16)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A16)</f>
         <v/>
       </c>
       <c r="F16" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A16,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A16,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G16" s="66">
@@ -42231,7 +42298,7 @@
         <v/>
       </c>
       <c r="J16" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A16,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A16,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K16" s="66">
@@ -42259,11 +42326,11 @@
         <v/>
       </c>
       <c r="E17" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A17)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A17)</f>
         <v/>
       </c>
       <c r="F17" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A17,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A17,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G17" s="66">
@@ -42279,7 +42346,7 @@
         <v/>
       </c>
       <c r="J17" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A17,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A17,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K17" s="66">
@@ -42307,11 +42374,11 @@
         <v/>
       </c>
       <c r="E18" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A18)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A18)</f>
         <v/>
       </c>
       <c r="F18" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A18,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A18,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G18" s="66">
@@ -42327,7 +42394,7 @@
         <v/>
       </c>
       <c r="J18" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A18,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A18,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K18" s="66">
@@ -42355,11 +42422,11 @@
         <v/>
       </c>
       <c r="E19" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A19)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A19)</f>
         <v/>
       </c>
       <c r="F19" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A19,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A19,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G19" s="66">
@@ -42375,7 +42442,7 @@
         <v/>
       </c>
       <c r="J19" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A19,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A19,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K19" s="66">
@@ -42403,11 +42470,11 @@
         <v/>
       </c>
       <c r="E20" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A20)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A20)</f>
         <v/>
       </c>
       <c r="F20" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A20,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A20,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G20" s="66">
@@ -42423,7 +42490,7 @@
         <v/>
       </c>
       <c r="J20" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A20,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A20,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K20" s="66">
@@ -42451,11 +42518,11 @@
         <v/>
       </c>
       <c r="E21" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A21)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A21)</f>
         <v/>
       </c>
       <c r="F21" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A21,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A21,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G21" s="66">
@@ -42471,7 +42538,7 @@
         <v/>
       </c>
       <c r="J21" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A21,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A21,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K21" s="66">
@@ -42499,11 +42566,11 @@
         <v/>
       </c>
       <c r="E22" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A22)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A22)</f>
         <v/>
       </c>
       <c r="F22" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A22,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A22,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G22" s="66">
@@ -42519,7 +42586,7 @@
         <v/>
       </c>
       <c r="J22" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A22,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A22,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K22" s="66">
@@ -42547,11 +42614,11 @@
         <v/>
       </c>
       <c r="E23" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A23)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A23)</f>
         <v/>
       </c>
       <c r="F23" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A23,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A23,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G23" s="66">
@@ -42567,7 +42634,7 @@
         <v/>
       </c>
       <c r="J23" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A23,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A23,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K23" s="66">
@@ -42595,11 +42662,11 @@
         <v/>
       </c>
       <c r="E24" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A24)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A24)</f>
         <v/>
       </c>
       <c r="F24" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A24,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A24,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G24" s="66">
@@ -42615,7 +42682,7 @@
         <v/>
       </c>
       <c r="J24" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A24,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A24,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K24" s="66">
@@ -42643,11 +42710,11 @@
         <v/>
       </c>
       <c r="E25" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A25)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A25)</f>
         <v/>
       </c>
       <c r="F25" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A25,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A25,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G25" s="66">
@@ -42663,7 +42730,7 @@
         <v/>
       </c>
       <c r="J25" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A25,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A25,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K25" s="66">
@@ -42691,11 +42758,11 @@
         <v/>
       </c>
       <c r="E26" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A26)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A26)</f>
         <v/>
       </c>
       <c r="F26" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A26,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A26,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G26" s="66">
@@ -42711,7 +42778,7 @@
         <v/>
       </c>
       <c r="J26" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A26,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A26,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K26" s="66">
@@ -42739,11 +42806,11 @@
         <v/>
       </c>
       <c r="E27" s="66">
-        <f>COUNTIF(Backlog!$M$2:$M$351,$A27)</f>
+        <f>COUNTIF(Backlog!$M$2:$M$352,$A27)</f>
         <v/>
       </c>
       <c r="F27" s="66">
-        <f>SUMIF(Backlog!$M$2:$M$351,$A27,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$M$2:$M$352,$A27,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="G27" s="66">
@@ -42759,7 +42826,7 @@
         <v/>
       </c>
       <c r="J27" s="66">
-        <f>COUNTIFS(Backlog!$M$2:$M$351,$A27,Backlog!$J$2:$J$351,"Must")</f>
+        <f>COUNTIFS(Backlog!$M$2:$M$352,$A27,Backlog!$J$2:$J$352,"Must")</f>
         <v/>
       </c>
       <c r="K27" s="66">
@@ -42974,11 +43041,11 @@
         </is>
       </c>
       <c r="C5" s="66">
-        <f>COUNTIF(Backlog!$H$2:$H$351,$A5)</f>
+        <f>COUNTIF(Backlog!$H$2:$H$352,$A5)</f>
         <v/>
       </c>
       <c r="D5" s="66">
-        <f>SUMIF(Backlog!$H$2:$H$351,$A5,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$H$2:$H$352,$A5,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="E5" s="74">
@@ -42990,11 +43057,11 @@
         <v/>
       </c>
       <c r="G5" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A5)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A5)</f>
         <v/>
       </c>
       <c r="H5" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A5)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A5)</f>
         <v/>
       </c>
     </row>
@@ -43010,11 +43077,11 @@
         </is>
       </c>
       <c r="C6" s="66">
-        <f>COUNTIF(Backlog!$H$2:$H$351,$A6)</f>
+        <f>COUNTIF(Backlog!$H$2:$H$352,$A6)</f>
         <v/>
       </c>
       <c r="D6" s="66">
-        <f>SUMIF(Backlog!$H$2:$H$351,$A6,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$H$2:$H$352,$A6,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="E6" s="74">
@@ -43026,11 +43093,11 @@
         <v/>
       </c>
       <c r="G6" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A6)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A6)</f>
         <v/>
       </c>
       <c r="H6" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A6)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A6)</f>
         <v/>
       </c>
     </row>
@@ -43046,11 +43113,11 @@
         </is>
       </c>
       <c r="C7" s="66">
-        <f>COUNTIF(Backlog!$H$2:$H$351,$A7)</f>
+        <f>COUNTIF(Backlog!$H$2:$H$352,$A7)</f>
         <v/>
       </c>
       <c r="D7" s="66">
-        <f>SUMIF(Backlog!$H$2:$H$351,$A7,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$H$2:$H$352,$A7,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="E7" s="74">
@@ -43062,11 +43129,11 @@
         <v/>
       </c>
       <c r="G7" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A7)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A7)</f>
         <v/>
       </c>
       <c r="H7" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A7)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A7)</f>
         <v/>
       </c>
     </row>
@@ -43082,11 +43149,11 @@
         </is>
       </c>
       <c r="C8" s="66">
-        <f>COUNTIF(Backlog!$H$2:$H$351,$A8)</f>
+        <f>COUNTIF(Backlog!$H$2:$H$352,$A8)</f>
         <v/>
       </c>
       <c r="D8" s="66">
-        <f>SUMIF(Backlog!$H$2:$H$351,$A8,Backlog!$L$2:$L$351)</f>
+        <f>SUMIF(Backlog!$H$2:$H$352,$A8,Backlog!$L$2:$L$352)</f>
         <v/>
       </c>
       <c r="E8" s="74">
@@ -43098,11 +43165,11 @@
         <v/>
       </c>
       <c r="G8" s="66">
-        <f>_xlfn.MINIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A8)</f>
+        <f>_xlfn.MINIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A8)</f>
         <v/>
       </c>
       <c r="H8" s="66">
-        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$351,Backlog!$H$2:$H$351,$A8)</f>
+        <f>_xlfn.MAXIFS(Backlog!$M$2:$M$352,Backlog!$H$2:$H$352,$A8)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(plan): mark E07 Clinic Setup tasks NB-060 to NB-070 as Done
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -8152,7 +8152,7 @@
       </c>
       <c r="R61" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S61" s="68" t="n"/>
@@ -8239,7 +8239,7 @@
       </c>
       <c r="R62" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S62" s="62" t="n"/>
@@ -8326,7 +8326,7 @@
       </c>
       <c r="R63" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S63" s="68" t="n"/>
@@ -8413,7 +8413,7 @@
       </c>
       <c r="R64" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S64" s="62" t="n"/>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="R65" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S65" s="68" t="n"/>
@@ -8587,7 +8587,7 @@
       </c>
       <c r="R66" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S66" s="62" t="n"/>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="R67" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S67" s="68" t="n"/>
@@ -8761,7 +8761,7 @@
       </c>
       <c r="R68" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S68" s="62" t="n"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="R69" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S69" s="68" t="n"/>
@@ -8935,7 +8935,7 @@
       </c>
       <c r="R70" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S70" s="62" t="n"/>
@@ -9022,7 +9022,7 @@
       </c>
       <c r="R71" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="S71" s="68" t="n"/>

</xml_diff>

<commit_message>
Mark partially-built E11/E12 tickets as In progress in the backlog
NB-105/106/107/108/109/115/116/121/122/127 each have a real, tested slice
shipped but don't meet their full stated acceptance criteria yet (see the
prior commit's message for the specific gaps per ticket) — In progress
reflects that more accurately than Not started or Done.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -12047,7 +12047,7 @@
       </c>
       <c r="R106" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S106" s="62" t="n"/>
@@ -12134,7 +12134,7 @@
       </c>
       <c r="R107" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S107" s="68" t="n"/>
@@ -12221,7 +12221,7 @@
       </c>
       <c r="R108" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S108" s="62" t="n"/>
@@ -12308,7 +12308,7 @@
       </c>
       <c r="R109" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S109" s="68" t="n"/>
@@ -12395,7 +12395,7 @@
       </c>
       <c r="R110" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S110" s="62" t="n"/>
@@ -12913,7 +12913,7 @@
       </c>
       <c r="R116" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S116" s="62" t="n"/>
@@ -13000,7 +13000,7 @@
       </c>
       <c r="R117" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S117" s="68" t="n"/>
@@ -13435,7 +13435,7 @@
       </c>
       <c r="R122" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S122" s="62" t="n"/>
@@ -13522,7 +13522,7 @@
       </c>
       <c r="R123" s="68" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S123" s="68" t="n"/>
@@ -13957,7 +13957,7 @@
       </c>
       <c r="R128" s="62" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="S128" s="62" t="n"/>

</xml_diff>

<commit_message>
Add NB-352: tenant provisioning console page, status Done
Backfilled — this ticket didn't exist before I built the page. E22's
provisioning cluster (NB-258/259/260/261) was all backend-only, and
NB-262 covers the separate Fleet screen, so nothing in the backlog ever
tracked the actual /platform/provisioning frontend. Filed to close that
gap now that it's built.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S353"/>
+  <dimension ref="A1:S354"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="50" min="1" max="1"/>
@@ -33204,6 +33204,85 @@
         <f>SUM(O2:O352)</f>
         <v/>
       </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="68" t="inlineStr">
+        <is>
+          <t>NB-352</t>
+        </is>
+      </c>
+      <c r="B354" s="68" t="inlineStr">
+        <is>
+          <t>E22 Platform Console — SaaS Operations</t>
+        </is>
+      </c>
+      <c r="C354" s="68" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D354" s="68" t="inlineStr">
+        <is>
+          <t>Tenant Provisioning console page</t>
+        </is>
+      </c>
+      <c r="E354" s="68" t="inlineStr">
+        <is>
+          <t>Frontend for the provisioning job queue (NB-258/259/260/261) — create a job, approve enterprise-gated jobs, advance and inspect each of the six steps with its status and error detail.</t>
+        </is>
+      </c>
+      <c r="F354" s="68" t="inlineStr">
+        <is>
+          <t>SSA-01</t>
+        </is>
+      </c>
+      <c r="G354" s="68" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="H354" s="68" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="I354" s="68" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="J354" s="69" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="K354" s="69" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L354" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="M354" s="69" t="n"/>
+      <c r="N354" s="68" t="n"/>
+      <c r="O354" s="70" t="n"/>
+      <c r="P354" s="68" t="inlineStr">
+        <is>
+          <t>NB-258, NB-259, NB-260, NB-261</t>
+        </is>
+      </c>
+      <c r="Q354" s="68" t="inlineStr">
+        <is>
+          <t>Every step is inspectable with its own status and error detail; enterprise-path jobs cannot advance before approval</t>
+        </is>
+      </c>
+      <c r="R354" s="68" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="S354" s="68" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S350"/>

</xml_diff>

<commit_message>
Add NB-353: provisioning creates the owner's real login and emails the invite
verify_invite_owner now creates a login-capable staff row for the owner
(reusing StaffService.invite/acceptInvite) instead of logging a mock line,
captures ownerMobile so the existing WhatsApp-OTP PIN reset works from day
one, and sends the invite link by real SMTP email (EmailSender seam:
SmtpEmailSender when SMTP_HOST is set, LoggingEmailSender otherwise). The
invite token is still also returned once on the advance() response as a
manual-relay fallback. Adds the missing /accept-invite/[token] page so the
link is actually usable.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S354"/>
+  <dimension ref="A1:S355"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="50" min="1" max="1"/>
@@ -33205,7 +33205,7 @@
         <v/>
       </c>
     </row>
-    <row r="354">
+    <row r="354" s="51">
       <c r="A354" s="68" t="inlineStr">
         <is>
           <t>NB-352</t>
@@ -33283,6 +33283,85 @@
         </is>
       </c>
       <c r="S354" s="68" t="n"/>
+    </row>
+    <row r="355" s="51">
+      <c r="A355" s="68" t="inlineStr">
+        <is>
+          <t>NB-353</t>
+        </is>
+      </c>
+      <c r="B355" s="68" t="inlineStr">
+        <is>
+          <t>E22 Platform Console — SaaS Operations</t>
+        </is>
+      </c>
+      <c r="C355" s="68" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D355" s="68" t="inlineStr">
+        <is>
+          <t>Provisioning creates the owner's real login</t>
+        </is>
+      </c>
+      <c r="E355" s="68" t="inlineStr">
+        <is>
+          <t>verify_invite_owner now creates a real, login-capable staff row for the owner (reusing StaffService.invite/acceptInvite) instead of logging a mock invite line. Captures ownerMobile at provisioning time so the existing WhatsApp-OTP PIN reset (AuthService.requestPinReset) works for this owner from day one. Sends the invite link by real email via Gmail SMTP (EmailSender seam: SmtpEmailSender when SMTP_HOST is configured, LoggingEmailSender otherwise — every local/test run today). The raw invite token is still also returned once on the advance() response as a manual-relay fallback if the email never lands.</t>
+        </is>
+      </c>
+      <c r="F355" s="68" t="inlineStr">
+        <is>
+          <t>SSA-01</t>
+        </is>
+      </c>
+      <c r="G355" s="68" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="H355" s="68" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="I355" s="68" t="inlineStr">
+        <is>
+          <t>Fullstack</t>
+        </is>
+      </c>
+      <c r="J355" s="69" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="K355" s="69" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="L355" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="M355" s="69" t="n"/>
+      <c r="N355" s="68" t="n"/>
+      <c r="O355" s="70" t="n"/>
+      <c r="P355" s="68" t="inlineStr">
+        <is>
+          <t>NB-258</t>
+        </is>
+      </c>
+      <c r="Q355" s="68" t="inlineStr">
+        <is>
+          <t>verify_invite_owner creates a staff row for the owner (status invited) with a hashed invite token; advance() returns the raw invite token exactly once, on the response immediately after that step runs; a fatal failure on a later step rolls back and deletes that staff row; retrying advance() after the owner is already invited does not create a duplicate row. When SMTP_HOST is configured, the owner also receives a real email containing the invite link.</t>
+        </is>
+      </c>
+      <c r="R355" s="68" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="S355" s="68" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S350"/>

</xml_diff>

<commit_message>
Add NB-357: platform-authored workflow templates replace owner flow editor
Phase 1 of the Arogya Fabric restructuring plan: an owner now picks one of a
published set of workflow templates (clinic_walkin, clinic_walkin_with_billing,
dental_procedure) per department and flips the toggles that template defines,
instead of freely reordering stages (NB-356). workflow_definitions +
department_workflow_selection replace visit_flow_steps; every existing
department is backfilled onto its closest matching template so live behavior
is unchanged. DepartmentService.resolveStatusSequence's external contract is
untouched, so QueueService/CheckoutService need no changes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S357"/>
+  <dimension ref="A1:S358"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="50" min="1" max="1"/>
@@ -33487,6 +33487,73 @@
         </is>
       </c>
       <c r="R357" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>NB-357</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>E10 Queue, Scheduling &amp; Availability</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Queue</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Platform-authored workflow templates replace owner-designed visit flow</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Phase 1 of the Arogya Fabric restructuring: replaces NB-356's freely-reorderable owner flow editor (visit_flow_steps) with a platform-authored template library (workflow_definitions: clinic_walkin, clinic_walkin_with_billing, dental_procedure) plus a small set of template-defined toggles (currently vitals_enabled). An owner now picks a published template per department and flips its toggles instead of reordering stages directly. department_workflow_selection replaces visit_flow_steps as the per-department row; DepartmentService.resolveStatusSequence (the single source of truth QueueService and CheckoutService both call) is re-pointed to the new tables with its external behavior unchanged. Every already-configured department is backfilled onto the closest matching platform template (or a one-off tenant-scoped snapshot template if nothing matches) so no tenant's live behavior changes.</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Owner,Reception,Nurse,Doctor,Billing</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>Clinic</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Fullstack</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="P358" t="inlineStr">
+        <is>
+          <t>NB-356</t>
+        </is>
+      </c>
+      <c r="Q358" t="inlineStr">
+        <is>
+          <t>GET /v1/departments/{id}/flow keeps returning the resolved, ordered step list unchanged for consult/checkout/nursing pages; an unconfigured department still falls back to vitals+consultation; POST /v1/departments/{id}/workflow accepts only a published templateCode plus toggles the chosen template defines, rejecting an unknown template code or a toggle the template does not define; the general-clinic and dental-clinic examples from NB-355/356 resolve identically when configured via clinic_walkin_with_billing and dental_procedure; the V40 migration backfill preserves every existing department's exact resolved sequence.</t>
+        </is>
+      </c>
+      <c r="R358" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
Add NB-358: additive org hierarchy + commercial axis schema (Arogya Fabric Phase 2)
V41 adds the architecture doc's org-hierarchy and commercial-axis columns/
tables on top of the confirmed mapping (owners=L1 Tenant, brands=L2 Brand,
tenants=L3 Facility, departments=L4 Department): tenants.facility_type and
billing_mode (defaulting to per_department to match NB-356's actual live
checkout behavior, not the doc's stated consolidated default), departments
.kind/specialty_code, and new RLS-isolated service_points/invoice_series
tables plus owner-scoped legal_entities/tax_registrations (no RLS, same
precedent as owners/brands themselves). Schema-only — nothing reads these
columns yet, so every existing tenant's behavior is unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S358"/>
+  <dimension ref="A1:S359"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="50" min="1" max="1"/>
@@ -33493,67 +33493,134 @@
       </c>
     </row>
     <row r="358">
-      <c r="A358" t="inlineStr">
+      <c r="A358" s="50" t="inlineStr">
         <is>
           <t>NB-357</t>
         </is>
       </c>
-      <c r="B358" t="inlineStr">
+      <c r="B358" s="50" t="inlineStr">
         <is>
           <t>E10 Queue, Scheduling &amp; Availability</t>
         </is>
       </c>
-      <c r="C358" t="inlineStr">
+      <c r="C358" s="50" t="inlineStr">
         <is>
           <t>Queue</t>
         </is>
       </c>
-      <c r="D358" t="inlineStr">
+      <c r="D358" s="50" t="inlineStr">
         <is>
           <t>Platform-authored workflow templates replace owner-designed visit flow</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr">
+      <c r="E358" s="50" t="inlineStr">
         <is>
           <t>Phase 1 of the Arogya Fabric restructuring: replaces NB-356's freely-reorderable owner flow editor (visit_flow_steps) with a platform-authored template library (workflow_definitions: clinic_walkin, clinic_walkin_with_billing, dental_procedure) plus a small set of template-defined toggles (currently vitals_enabled). An owner now picks a published template per department and flips its toggles instead of reordering stages directly. department_workflow_selection replaces visit_flow_steps as the per-department row; DepartmentService.resolveStatusSequence (the single source of truth QueueService and CheckoutService both call) is re-pointed to the new tables with its external behavior unchanged. Every already-configured department is backfilled onto the closest matching platform template (or a one-off tenant-scoped snapshot template if nothing matches) so no tenant's live behavior changes.</t>
         </is>
       </c>
-      <c r="G358" t="inlineStr">
+      <c r="G358" s="50" t="inlineStr">
         <is>
           <t>Owner,Reception,Nurse,Doctor,Billing</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr">
+      <c r="H358" s="50" t="inlineStr">
         <is>
           <t>Clinic</t>
         </is>
       </c>
-      <c r="I358" t="inlineStr">
+      <c r="I358" s="50" t="inlineStr">
         <is>
           <t>Fullstack</t>
         </is>
       </c>
-      <c r="J358" t="inlineStr">
+      <c r="J358" s="50" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="K358" t="inlineStr">
+      <c r="K358" s="50" t="inlineStr">
         <is>
           <t>MVP</t>
         </is>
       </c>
-      <c r="P358" t="inlineStr">
+      <c r="P358" s="50" t="inlineStr">
         <is>
           <t>NB-356</t>
         </is>
       </c>
-      <c r="Q358" t="inlineStr">
+      <c r="Q358" s="50" t="inlineStr">
         <is>
           <t>GET /v1/departments/{id}/flow keeps returning the resolved, ordered step list unchanged for consult/checkout/nursing pages; an unconfigured department still falls back to vitals+consultation; POST /v1/departments/{id}/workflow accepts only a published templateCode plus toggles the chosen template defines, rejecting an unknown template code or a toggle the template does not define; the general-clinic and dental-clinic examples from NB-355/356 resolve identically when configured via clinic_walkin_with_billing and dental_procedure; the V40 migration backfill preserves every existing department's exact resolved sequence.</t>
         </is>
       </c>
-      <c r="R358" t="inlineStr">
+      <c r="R358" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>NB-358</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>E01 Foundation &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Org hierarchy + commercial axis: additive schema (Arogya Fabric Phase 2)</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Phase 2 of the Arogya Fabric restructuring: additive-only schema from the architecture doc's org hierarchy and commercial axis (S6.3), confirmed against the current model (owners=L1 Tenant, brands=L2 Brand, tenants=L3 Facility, departments=L4 Department -- no isolation-grain change). Adds tenants.facility_type (clinic/single_specialty/multi_specialty) and tenants.billing_mode (defaults to per_department, matching NB-356's actual live checkout behaviour rather than the doc's stated consolidated default); departments.kind and specialty_code; new tenant-scoped, RLS-isolated service_points (L5) and invoice_series tables; new legal_entities/tax_registrations tables scoped by owner_id with no RLS of their own, matching the existing owners/brands precedent (V6). No application code reads any of this yet -- schema only, ahead of the feature that will need it.</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Platform,Owner</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>Post-MVP</t>
+        </is>
+      </c>
+      <c r="P359" t="inlineStr">
+        <is>
+          <t>NB-357</t>
+        </is>
+      </c>
+      <c r="Q359" t="inlineStr">
+        <is>
+          <t>Every already-provisioned tenant defaults to facility_type=clinic, billing_mode=per_department, and its default department to kind=clinical after the migration; service_points and invoice_series rows are only visible within the tenant session that created them (RLS), verified by OrgHierarchySchemaTest; legal_entities/tax_registrations/invoice_series form the doc's Legal Entity -&gt; Tax Registration -&gt; Invoice Series chain with a facility able to reference a tax registration via tenants.tax_registration_id.</t>
+        </is>
+      </c>
+      <c r="R359" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
Add NB-359: activate the dormant accessible_tenant_ids GUC (Arogya Fabric Phase 3)
V42 adds brands.data_visibility_scope (FACILITY default / BRAND / TENANT).
TenantContext.set() — called on every service method before any RLS-protected
query — now also computes app.accessible_tenant_ids fresh from the active
tenant's brand scope on every call, so the tenant_isolation policies V6
already patched with the accessible_tenant_ids OR clause start working with
zero further policy changes. FACILITY scope (the default, and any tenant
with no brand) resolves to no siblings, so this is a no-op for every tenant
today — no UI lets an owner change the scope yet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S359"/>
+  <dimension ref="A1:S360"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="50" min="1" max="1"/>
@@ -33560,67 +33560,134 @@
       </c>
     </row>
     <row r="359">
-      <c r="A359" t="inlineStr">
+      <c r="A359" s="50" t="inlineStr">
         <is>
           <t>NB-358</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B359" s="50" t="inlineStr">
         <is>
           <t>E01 Foundation &amp; Architecture</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr">
+      <c r="C359" s="50" t="inlineStr">
         <is>
           <t>Architecture</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr">
+      <c r="D359" s="50" t="inlineStr">
         <is>
           <t>Org hierarchy + commercial axis: additive schema (Arogya Fabric Phase 2)</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr">
+      <c r="E359" s="50" t="inlineStr">
         <is>
           <t>Phase 2 of the Arogya Fabric restructuring: additive-only schema from the architecture doc's org hierarchy and commercial axis (S6.3), confirmed against the current model (owners=L1 Tenant, brands=L2 Brand, tenants=L3 Facility, departments=L4 Department -- no isolation-grain change). Adds tenants.facility_type (clinic/single_specialty/multi_specialty) and tenants.billing_mode (defaults to per_department, matching NB-356's actual live checkout behaviour rather than the doc's stated consolidated default); departments.kind and specialty_code; new tenant-scoped, RLS-isolated service_points (L5) and invoice_series tables; new legal_entities/tax_registrations tables scoped by owner_id with no RLS of their own, matching the existing owners/brands precedent (V6). No application code reads any of this yet -- schema only, ahead of the feature that will need it.</t>
         </is>
       </c>
-      <c r="G359" t="inlineStr">
+      <c r="G359" s="50" t="inlineStr">
         <is>
           <t>Platform,Owner</t>
         </is>
       </c>
-      <c r="H359" t="inlineStr">
+      <c r="H359" s="50" t="inlineStr">
         <is>
           <t>Shared</t>
         </is>
       </c>
-      <c r="I359" t="inlineStr">
+      <c r="I359" s="50" t="inlineStr">
         <is>
           <t>Architecture</t>
         </is>
       </c>
-      <c r="J359" t="inlineStr">
+      <c r="J359" s="50" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="K359" t="inlineStr">
+      <c r="K359" s="50" t="inlineStr">
         <is>
           <t>Post-MVP</t>
         </is>
       </c>
-      <c r="P359" t="inlineStr">
+      <c r="P359" s="50" t="inlineStr">
         <is>
           <t>NB-357</t>
         </is>
       </c>
-      <c r="Q359" t="inlineStr">
+      <c r="Q359" s="50" t="inlineStr">
         <is>
           <t>Every already-provisioned tenant defaults to facility_type=clinic, billing_mode=per_department, and its default department to kind=clinical after the migration; service_points and invoice_series rows are only visible within the tenant session that created them (RLS), verified by OrgHierarchySchemaTest; legal_entities/tax_registrations/invoice_series form the doc's Legal Entity -&gt; Tax Registration -&gt; Invoice Series chain with a facility able to reference a tax registration via tenants.tax_registration_id.</t>
         </is>
       </c>
-      <c r="R359" t="inlineStr">
+      <c r="R359" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="50" t="inlineStr">
+        <is>
+          <t>NB-359</t>
+        </is>
+      </c>
+      <c r="B360" s="50" t="inlineStr">
+        <is>
+          <t>E01 Foundation &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="C360" s="50" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="D360" s="50" t="inlineStr">
+        <is>
+          <t>Cross-facility data visibility: activate the dormant accessible_tenant_ids GUC (Arogya Fabric Phase 3)</t>
+        </is>
+      </c>
+      <c r="E360" s="50" t="inlineStr">
+        <is>
+          <t>Phase 3 of the Arogya Fabric restructuring: adds brands.data_visibility_scope (FACILITY default / BRAND / TENANT, the doc's S6.3 brand-visibility model) and wires TenantContext.set() -- called on every service method before any RLS-protected query -- to compute app.accessible_tenant_ids fresh from the active tenant's brand scope on every call. Every tenant_isolation policy V6 already patched with the OR tenant_id::text = ANY(accessible_tenant_ids) clause picks this up with zero further changes. FACILITY scope (the default, and any tenant with no brand) resolves to no siblings at all, so this is a no-op for every tenant today; no UI or endpoint yet lets an owner change the scope.</t>
+        </is>
+      </c>
+      <c r="G360" s="50" t="inlineStr">
+        <is>
+          <t>Platform,Owner</t>
+        </is>
+      </c>
+      <c r="H360" s="50" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="I360" s="50" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="J360" s="50" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="K360" s="50" t="inlineStr">
+        <is>
+          <t>Post-MVP</t>
+        </is>
+      </c>
+      <c r="P360" s="50" t="inlineStr">
+        <is>
+          <t>NB-358</t>
+        </is>
+      </c>
+      <c r="Q360" s="50" t="inlineStr">
+        <is>
+          <t>A tenant with no brand, or a brand at the default FACILITY scope, sees exactly the same rows as before this change on every V6-patched table; a brand set to BRAND scope makes every sibling facility under that brand mutually visible on those tables; a brand set to TENANT scope extends that to every facility across every brand of the same owner; an unrelated brand under the same or a different owner never leaks in; a scope change takes effect on the very next request with no session/cache invalidation needed, verified end-to-end by CrossFacilityVisibilityTest.</t>
+        </is>
+      </c>
+      <c r="R360" s="50" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
Add NB-360: encounter identity + fixed stage vocabulary (Arogya Fabric Phase 4)
V43 begins reconciling queue_entries toward the architecture doc's ENCOUNTER/
ENCOUNTER_SEGMENT model without a physical table split — it's FK-referenced
by clinical_notes, invoices, prescriptions and procedure_orders, so a split
would be a large, risky rewrite for a doc-fidelity win nothing built so far
needs. Instead queue_entries (one row per department leg = an
ENCOUNTER_SEGMENT) gains encounter_id (shared by every leg of one visit,
defaulted by a BEFORE INSERT trigger), class, current_stage (the doc's fixed
S9.1 vocabulary, computed from status by a SQL function + trigger), and
workflow_definition_id (resolved from department_workflow_selection at
insert) — all DB-managed so no Java call site can drift out of sync.
QueueService.transfer() propagates encounter_id onto the new leg; everything
else is trigger-driven.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nabd HMS - Implementation Task Plan v2.xlsx
+++ b/Nabd HMS - Implementation Task Plan v2.xlsx
@@ -2929,7 +2929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S360"/>
+  <dimension ref="A1:S361"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="50" min="1" max="1"/>
@@ -33688,6 +33688,73 @@
         </is>
       </c>
       <c r="R360" s="50" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>NB-360</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>E10 Queue, Scheduling &amp; Availability</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Queue</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Encounter identity + fixed stage vocabulary on queue_entries (Arogya Fabric Phase 4)</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Phase 4 of the Arogya Fabric restructuring: begins reconciling queue_entries toward the architecture doc's ENCOUNTER/ENCOUNTER_SEGMENT model (S6.5) without a physical table split -- queue_entries is FK-referenced by clinical_notes, invoices, prescriptions and procedure_orders (V19-V29), so splitting it now would be a large, risky rewrite for a doc-fidelity win nothing built so far needs. Instead queue_entries stays one row per department leg (an ENCOUNTER_SEGMENT) and gains: encounter_id (self-referencing, shared by every leg of one visit, defaulted by a BEFORE INSERT trigger so no Java call site can forget it), class (ambulatory/procedure/teleconsult/inpatient, always ambulatory today), current_stage (the doc's fixed S9.1 stage vocabulary, computed from status by a SQL function + trigger so dashboards can key off a stable set of stages regardless of a department's configured step names), and workflow_definition_id (the platform template governing this leg, resolved from department_workflow_selection at insert). All three triggers/functions are the single source of truth -- no Java-side duplicate of the status-to-stage mapping.</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>Owner,Reception,Nurse,Doctor,Billing</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>Clinic</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Fullstack</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>Post-MVP</t>
+        </is>
+      </c>
+      <c r="P361" t="inlineStr">
+        <is>
+          <t>NB-359</t>
+        </is>
+      </c>
+      <c r="Q361" t="inlineStr">
+        <is>
+          <t>A fresh check-in gets encounter_id equal to its own id, class=ambulatory, and current_stage=CHECKED_IN; a transfer propagates the original encounter_id onto the new leg and the closed leg's current_stage becomes COMPLETED; every subsequent status PATCH keeps current_stage in sync automatically; workflow_definition_id is null for an unconfigured department and set to the selected template once one is chosen; every existing row is correctly backfilled by the migration.</t>
+        </is>
+      </c>
+      <c r="R361" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>